<commit_message>
WIP P12e: medición según cotización, enlace de stock al importar, cotización sin bloqueo de taller
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/tests/e2e/fixtures/p12-pro6004-compras.xlsx
+++ b/frontend/tests/e2e/fixtures/p12-pro6004-compras.xlsx
@@ -5220,13 +5220,21 @@
       <c r="G5" s="15" t="inlineStr"/>
       <c r="H5" s="15" t="inlineStr"/>
       <c r="I5" s="15" t="inlineStr"/>
-      <c r="J5" s="15" t="inlineStr"/>
+      <c r="J5" s="15" t="inlineStr">
+        <is>
+          <t>20.00</t>
+        </is>
+      </c>
       <c r="K5" s="15" t="inlineStr"/>
       <c r="L5" s="15" t="inlineStr"/>
       <c r="M5" s="15" t="inlineStr"/>
       <c r="N5" s="15" t="inlineStr"/>
       <c r="O5" s="15" t="inlineStr"/>
-      <c r="P5" s="15" t="inlineStr"/>
+      <c r="P5" s="15" t="inlineStr">
+        <is>
+          <t>2.60</t>
+        </is>
+      </c>
       <c r="Q5" s="15" t="inlineStr"/>
       <c r="R5" s="15" t="inlineStr"/>
       <c r="S5" s="15" t="inlineStr"/>
@@ -5280,7 +5288,7 @@
       </c>
       <c r="AF5" s="15" t="inlineStr">
         <is>
-          <t>OT 385 del taller (NuveraPro, 29-10-2025), págs. 1, 6 y 7</t>
+          <t>OT 385 del taller (NuveraPro, 29-10-2025), págs. 1, 6 y 7; peso y área máxima: ficha de vidrio del taller de ensayo</t>
         </is>
       </c>
     </row>

</xml_diff>